<commit_message>
Reprioritize hiring waves on Kathy-tab weights
Waves now ranked by Kathy score (MDs/Rep 20% / Clinics/Rep 60% / Women 10% /
Income 10%); Hire Wave column added to Kathy tab, mirrored on Territory Plan.
Territory Plan score kept as reference only. Waves cumulate 9/15/23/28.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ysekWyVFey7vTLxxqcMoX
</commit_message>
<xml_diff>
--- a/docs/deliverables/Femasys_Territory_Plan_v4.xlsx
+++ b/docs/deliverables/Femasys_Territory_Plan_v4.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="248">
   <si>
     <t xml:space="preserve">FemaSeed U.S. Territory Plan — v4 (ALL-MD Universe, 28-Rep Hard Cap)</t>
   </si>
@@ -81,10 +81,10 @@
     <t xml:space="preserve">No source provides volume for the full ALL-MD universe (row-level volume exists only for the &gt;=10 subset), so v3's 15% volume weight is redistributed proportionally rather than reusing partial-coverage volume.</t>
   </si>
   <si>
-    <t xml:space="preserve">Weights: All MDs 47.06% / All Clinics 29.41% / Women 25-44 11.76% / Income 11.76% (= 40/25/10/10 renormalized over 85). Each component scored as share of territory maximum, weighted, rescaled to 0-100 max. Education retained for reference at 0%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Result vs v3: 18 of 25 rankings changed. Top 8: CA-HI, TX, NY, PA-NJ, FL, New England, WA-OR-AK, IL.</t>
+    <t xml:space="preserve">Reference score (Territory Plan tab, rep-independent): All MDs 47.06% / All Clinics 29.41% / Women 25-44 11.76% / Income 11.76% (= 40/25/10/10 renormalized over 85), share-of-max method. Retained for reference; it does NOT drive prioritization.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRIORITIZATION uses the Kathy - ALL Universe score (per Rajiv, 2026-07-22): All MDs/Rep 20% / All Clinics/Rep 60% / Women 25-44 10% / Median Income 10% / Education 0%, min-max normalized 0-100 across staffed territories. Top 8: CA-HI, New England, TX, IL, WA-OR-AK, GA, AZ-NV-ID-MT, MI. Because components are per-rep, ranks depend on the rep allocation.</t>
   </si>
   <si>
     <t xml:space="preserve">KATHY - ALL UNIVERSE TAB</t>
@@ -96,7 +96,7 @@
     <t xml:space="preserve">HIRING WAVES</t>
   </si>
   <si>
-    <t xml:space="preserve">Territories ranked by v4 score, wave sizes 7/5/7/6. Cumulative reps 12 / 17 / 24 / 28. Wave 4 includes the two unstaffed territories at 0 reps.</t>
+    <t xml:space="preserve">Territories ranked by the Kathy - ALL Universe score, wave sizes 7/5/7/6. Cumulative reps 9 / 15 / 23 / 28. Wave 4 includes the two unstaffed territories at 0 reps. Wave membership recalculates from the Kathy tab if reps are edited (lists in column B are a snapshot).</t>
   </si>
   <si>
     <t xml:space="preserve">STRATEGIC CAVEAT — MANDATE STATES (carried from v3, still open): rankings are pure opportunity, not mandate-adjusted. Northeast (incl. mandate states) remains in early waves. Verify the current mandate list and re-sequence before committing hires — statuses have changed recently.</t>
@@ -462,7 +462,7 @@
     <t xml:space="preserve">Rank Change</t>
   </si>
   <si>
-    <t xml:space="preserve">Hire Wave (v4)</t>
+    <t xml:space="preserve">Hire Wave (Kathy weights)</t>
   </si>
   <si>
     <t xml:space="preserve">Houston, Dallas, Austin</t>
@@ -579,7 +579,7 @@
     <t xml:space="preserve">Greenville, Florence, Spartanburg</t>
   </si>
   <si>
-    <t xml:space="preserve">HARD CAP: 28 reps. Allocation (blue, adjustable — keep the column total at 28): 2 reps each for TX, CA-HI, NY, FL, PA-NJ; 1 rep for 18 territories; 0 reps for T24 IA-SD-ND-WY and T25 SC (unstaffed at the cap). Per-rep loads, Score, Rank, and Hiring Wave figures recalculate. Against the ALL-MD universe (18,405) the 28 reps average ~657 MDs each — use with the &gt;=10 / &gt;=20 tiers on State Market Summary as a prioritization model. Women 25-44 and Wtd Income carried from v3 unchanged (blue = input). Score v4 weights: All MDs 47.06% / All Clinics 29.41% / Women 25-44 11.76% / Income 11.76% (see Read Me). Score does not depend on Reps.</t>
+    <t xml:space="preserve">HARD CAP: 28 reps. Allocation (blue, adjustable — keep the column total at 28): 2 reps each for TX, CA-HI, NY, FL, PA-NJ; 1 rep for 18 territories; 0 reps for T24 IA-SD-ND-WY and T25 SC (unstaffed at the cap). Per-rep loads and dependent figures recalculate. PRIORITIZATION: hiring waves are driven by the Kathy - ALL Universe score/rank (per-rep weights 20/60/10/10); the Score v4 column here (market-size weights, rep-independent) is retained for reference only. Against the ALL-MD universe (18,405) the 28 reps average ~657 MDs each — use with the &gt;=10 / &gt;=20 tiers on State Market Summary as a prioritization model. Women 25-44 and Wtd Income carried from v3 unchanged (blue = input).</t>
   </si>
   <si>
     <t xml:space="preserve">Wave</t>
@@ -600,16 +600,16 @@
     <t xml:space="preserve">Wave 1</t>
   </si>
   <si>
-    <t xml:space="preserve">T02 CA-HI; T01 TX; T03 NY; T06 PA-NJ; T05 FL; T08 MA-CT-NH-ME-VT-RI; T12 WA-OR-AK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Highest v4 opportunity; staff first</t>
+    <t xml:space="preserve">T02 CA-HI; T08 MA-CT-NH-ME-VT-RI; T01 TX; T17 IL; T12 WA-OR-AK; T11 GA; T15 AZ-NV-ID-MT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Highest Kathy-weighted score; staff first</t>
   </si>
   <si>
     <t xml:space="preserve">Wave 2</t>
   </si>
   <si>
-    <t xml:space="preserve">T17 IL; T09 MN-WI; T04 OH; T07 MI; T13 NC</t>
+    <t xml:space="preserve">T07 MI; T03 NY; T09 MN-WI; T04 OH; T13 NC</t>
   </si>
   <si>
     <t xml:space="preserve">Second tier</t>
@@ -618,7 +618,7 @@
     <t xml:space="preserve">Wave 3</t>
   </si>
   <si>
-    <t xml:space="preserve">T11 GA; T15 AZ-NV-ID-MT; T10 MO-KY; T16 CO-UT; T14 KS-OK-NE-NM; T22 MD-WV-DE-DC; T21 VA</t>
+    <t xml:space="preserve">T10 MO-KY; T16 CO-UT; T14 KS-OK-NE-NM; T06 PA-NJ; T22 MD-WV-DE-DC; T21 VA; T19 LA-AR</t>
   </si>
   <si>
     <t xml:space="preserve">Regional completion</t>
@@ -627,16 +627,16 @@
     <t xml:space="preserve">Wave 4</t>
   </si>
   <si>
-    <t xml:space="preserve">T19 LA-AR; T18 AL-MS; T20 IN; T23 TN; T24 IA-SD-ND-WY; T25 SC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full national at the 28 cap</t>
+    <t xml:space="preserve">T18 AL-MS; T05 FL; T23 TN; T20 IN; T24 IA-SD-ND-WY (0 reps); T25 SC (0 reps)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balance of the 28; includes the two unstaffed territories</t>
   </si>
   <si>
     <t xml:space="preserve">CAVEAT: rankings are pure opportunity, not mandate-adjusted. Northeast (incl. mandate states) remains in early waves under v3 weights. Verify the current mandate list (Phase 2) and re-sequence before committing hires.</t>
   </si>
   <si>
-    <t xml:space="preserve">v4 notes: waves ranked by v4 score, wave sizes 7/5/7/6 territories. Rep counts use the hard 28-cap allocation (2 each: TX, CA-HI, NY, FL, PA-NJ; 1 each: 18 territories). Wave 4 lists T24 IA-SD-ND-WY and T25 SC at 0 reps — unstaffed at the cap. Cumulative total = 28.</t>
+    <t xml:space="preserve">v4 notes: waves ranked by the Kathy - ALL Universe score (All MDs/Rep 20% / All Clinics/Rep 60% / Women 25-44 10% / Median Income 10%), wave sizes 7/5/7/6. Rep counts use the hard 28-cap allocation (2 each: TX, CA-HI, NY, FL, PA-NJ; 1 each: 18 territories). Wave 4 lists T24 IA-SD-ND-WY and T25 SC at 0 reps — unstaffed at the cap. Cumulative total = 28. NOTE: because the score weights per-rep load, editing the Reps column re-shuffles ranks and wave membership; the wave lists in column B are a snapshot of the current allocation — re-check after any rep change.</t>
   </si>
   <si>
     <t xml:space="preserve">Kathy - ALL Universe: all counts sum Waterfall A rev1 labeled columns only (via State Market Summary). Reps (J, blue) = the 28-rep hard-cap allocation (2 each: TX, CA-HI, NY, FL, PA-NJ; 1 each: 18 territories; 0: IA-SD-ND-WY, SC) — overwrite freely, keep total 28; per-rep loads, Academic Share, Score, and Rank recalculate. Unstaffed territories show no per-rep figures or score.</t>
@@ -688,6 +688,9 @@
   </si>
   <si>
     <t xml:space="preserve">Rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hire Wave</t>
   </si>
   <si>
     <t xml:space="preserve">T01 TX</t>
@@ -772,13 +775,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="\$#,##0"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="0.0%"/>
+    <numFmt numFmtId="170" formatCode="General"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -922,7 +926,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1040,6 +1044,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5141,7 +5149,7 @@
         <v>-1</v>
       </c>
       <c r="O2" s="7" t="n">
-        <f aca="false">IF(L2&lt;=7,1,IF(L2&lt;=12,2,IF(L2&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S4</f>
         <v>1</v>
       </c>
     </row>
@@ -5196,7 +5204,7 @@
         <v>1</v>
       </c>
       <c r="O3" s="7" t="n">
-        <f aca="false">IF(L3&lt;=7,1,IF(L3&lt;=12,2,IF(L3&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S5</f>
         <v>1</v>
       </c>
     </row>
@@ -5251,8 +5259,8 @@
         <v>0</v>
       </c>
       <c r="O4" s="7" t="n">
-        <f aca="false">IF(L4&lt;=7,1,IF(L4&lt;=12,2,IF(L4&lt;=19,3,4)))</f>
-        <v>1</v>
+        <f aca="false">'Kathy - ALL Universe'!S6</f>
+        <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5306,7 +5314,7 @@
         <v>-6</v>
       </c>
       <c r="O5" s="7" t="n">
-        <f aca="false">IF(L5&lt;=7,1,IF(L5&lt;=12,2,IF(L5&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S7</f>
         <v>2</v>
       </c>
     </row>
@@ -5361,8 +5369,8 @@
         <v>0</v>
       </c>
       <c r="O6" s="7" t="n">
-        <f aca="false">IF(L6&lt;=7,1,IF(L6&lt;=12,2,IF(L6&lt;=19,3,4)))</f>
-        <v>1</v>
+        <f aca="false">'Kathy - ALL Universe'!S8</f>
+        <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5416,8 +5424,8 @@
         <v>2</v>
       </c>
       <c r="O7" s="7" t="n">
-        <f aca="false">IF(L7&lt;=7,1,IF(L7&lt;=12,2,IF(L7&lt;=19,3,4)))</f>
-        <v>1</v>
+        <f aca="false">'Kathy - ALL Universe'!S9</f>
+        <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5471,7 +5479,7 @@
         <v>-4</v>
       </c>
       <c r="O8" s="7" t="n">
-        <f aca="false">IF(L8&lt;=7,1,IF(L8&lt;=12,2,IF(L8&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S10</f>
         <v>2</v>
       </c>
     </row>
@@ -5526,7 +5534,7 @@
         <v>2</v>
       </c>
       <c r="O9" s="7" t="n">
-        <f aca="false">IF(L9&lt;=7,1,IF(L9&lt;=12,2,IF(L9&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S11</f>
         <v>1</v>
       </c>
     </row>
@@ -5581,7 +5589,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="7" t="n">
-        <f aca="false">IF(L10&lt;=7,1,IF(L10&lt;=12,2,IF(L10&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S12</f>
         <v>2</v>
       </c>
     </row>
@@ -5636,7 +5644,7 @@
         <v>-5</v>
       </c>
       <c r="O11" s="7" t="n">
-        <f aca="false">IF(L11&lt;=7,1,IF(L11&lt;=12,2,IF(L11&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S13</f>
         <v>3</v>
       </c>
     </row>
@@ -5691,8 +5699,8 @@
         <v>-2</v>
       </c>
       <c r="O12" s="7" t="n">
-        <f aca="false">IF(L12&lt;=7,1,IF(L12&lt;=12,2,IF(L12&lt;=19,3,4)))</f>
-        <v>3</v>
+        <f aca="false">'Kathy - ALL Universe'!S14</f>
+        <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5746,7 +5754,7 @@
         <v>5</v>
       </c>
       <c r="O13" s="7" t="n">
-        <f aca="false">IF(L13&lt;=7,1,IF(L13&lt;=12,2,IF(L13&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S15</f>
         <v>1</v>
       </c>
     </row>
@@ -5801,7 +5809,7 @@
         <v>1</v>
       </c>
       <c r="O14" s="7" t="n">
-        <f aca="false">IF(L14&lt;=7,1,IF(L14&lt;=12,2,IF(L14&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S16</f>
         <v>2</v>
       </c>
     </row>
@@ -5856,7 +5864,7 @@
         <v>-3</v>
       </c>
       <c r="O15" s="7" t="n">
-        <f aca="false">IF(L15&lt;=7,1,IF(L15&lt;=12,2,IF(L15&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S17</f>
         <v>3</v>
       </c>
     </row>
@@ -5911,8 +5919,8 @@
         <v>1</v>
       </c>
       <c r="O16" s="7" t="n">
-        <f aca="false">IF(L16&lt;=7,1,IF(L16&lt;=12,2,IF(L16&lt;=19,3,4)))</f>
-        <v>3</v>
+        <f aca="false">'Kathy - ALL Universe'!S18</f>
+        <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5966,7 +5974,7 @@
         <v>0</v>
       </c>
       <c r="O17" s="7" t="n">
-        <f aca="false">IF(L17&lt;=7,1,IF(L17&lt;=12,2,IF(L17&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S19</f>
         <v>3</v>
       </c>
     </row>
@@ -6021,8 +6029,8 @@
         <v>9</v>
       </c>
       <c r="O18" s="7" t="n">
-        <f aca="false">IF(L18&lt;=7,1,IF(L18&lt;=12,2,IF(L18&lt;=19,3,4)))</f>
-        <v>2</v>
+        <f aca="false">'Kathy - ALL Universe'!S20</f>
+        <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6076,7 +6084,7 @@
         <v>-3</v>
       </c>
       <c r="O19" s="7" t="n">
-        <f aca="false">IF(L19&lt;=7,1,IF(L19&lt;=12,2,IF(L19&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S21</f>
         <v>4</v>
       </c>
     </row>
@@ -6131,8 +6139,8 @@
         <v>-1</v>
       </c>
       <c r="O20" s="7" t="n">
-        <f aca="false">IF(L20&lt;=7,1,IF(L20&lt;=12,2,IF(L20&lt;=19,3,4)))</f>
-        <v>4</v>
+        <f aca="false">'Kathy - ALL Universe'!S22</f>
+        <v>3</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6186,7 +6194,7 @@
         <v>-2</v>
       </c>
       <c r="O21" s="7" t="n">
-        <f aca="false">IF(L21&lt;=7,1,IF(L21&lt;=12,2,IF(L21&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S23</f>
         <v>4</v>
       </c>
     </row>
@@ -6241,7 +6249,7 @@
         <v>2</v>
       </c>
       <c r="O22" s="7" t="n">
-        <f aca="false">IF(L22&lt;=7,1,IF(L22&lt;=12,2,IF(L22&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S24</f>
         <v>3</v>
       </c>
     </row>
@@ -6296,7 +6304,7 @@
         <v>4</v>
       </c>
       <c r="O23" s="7" t="n">
-        <f aca="false">IF(L23&lt;=7,1,IF(L23&lt;=12,2,IF(L23&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S25</f>
         <v>3</v>
       </c>
     </row>
@@ -6351,7 +6359,7 @@
         <v>0</v>
       </c>
       <c r="O24" s="7" t="n">
-        <f aca="false">IF(L24&lt;=7,1,IF(L24&lt;=12,2,IF(L24&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S26</f>
         <v>4</v>
       </c>
     </row>
@@ -6406,7 +6414,7 @@
         <v>0</v>
       </c>
       <c r="O25" s="7" t="n">
-        <f aca="false">IF(L25&lt;=7,1,IF(L25&lt;=12,2,IF(L25&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S27</f>
         <v>4</v>
       </c>
     </row>
@@ -6461,7 +6469,7 @@
         <v>0</v>
       </c>
       <c r="O26" s="7" t="n">
-        <f aca="false">IF(L26&lt;=7,1,IF(L26&lt;=12,2,IF(L26&lt;=19,3,4)))</f>
+        <f aca="false">'Kathy - ALL Universe'!S28</f>
         <v>4</v>
       </c>
     </row>
@@ -6575,12 +6583,12 @@
         <v>191</v>
       </c>
       <c r="C2" s="8" t="n">
-        <f aca="false">SUMIF('Territory Plan'!$O$2:$O$26,1,'Territory Plan'!$F$2:$F$26)</f>
-        <v>12</v>
+        <f aca="false">SUMIF('Kathy - ALL Universe'!$S$4:$S$28,1,'Kathy - ALL Universe'!$J$4:$J$28)</f>
+        <v>9</v>
       </c>
       <c r="D2" s="8" t="n">
         <f aca="false">SUM($C$2:$C2)</f>
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>192</v>
@@ -6594,12 +6602,12 @@
         <v>194</v>
       </c>
       <c r="C3" s="8" t="n">
-        <f aca="false">SUMIF('Territory Plan'!$O$2:$O$26,2,'Territory Plan'!$F$2:$F$26)</f>
-        <v>5</v>
+        <f aca="false">SUMIF('Kathy - ALL Universe'!$S$4:$S$28,2,'Kathy - ALL Universe'!$J$4:$J$28)</f>
+        <v>6</v>
       </c>
       <c r="D3" s="8" t="n">
         <f aca="false">SUM($C$2:$C3)</f>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>195</v>
@@ -6613,12 +6621,12 @@
         <v>197</v>
       </c>
       <c r="C4" s="8" t="n">
-        <f aca="false">SUMIF('Territory Plan'!$O$2:$O$26,3,'Territory Plan'!$F$2:$F$26)</f>
-        <v>7</v>
+        <f aca="false">SUMIF('Kathy - ALL Universe'!$S$4:$S$28,3,'Kathy - ALL Universe'!$J$4:$J$28)</f>
+        <v>8</v>
       </c>
       <c r="D4" s="8" t="n">
         <f aca="false">SUM($C$2:$C4)</f>
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>198</v>
@@ -6632,8 +6640,8 @@
         <v>200</v>
       </c>
       <c r="C5" s="8" t="n">
-        <f aca="false">SUMIF('Territory Plan'!$O$2:$O$26,4,'Territory Plan'!$F$2:$F$26)</f>
-        <v>4</v>
+        <f aca="false">SUMIF('Kathy - ALL Universe'!$S$4:$S$28,4,'Kathy - ALL Universe'!$J$4:$J$28)</f>
+        <v>5</v>
       </c>
       <c r="D5" s="8" t="n">
         <f aca="false">SUM($C$2:$C5)</f>
@@ -6681,7 +6689,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="E1:R31"/>
+  <dimension ref="E1:S31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20"/>
@@ -6694,6 +6702,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6777,10 +6786,13 @@
       <c r="R3" s="16" t="s">
         <v>220</v>
       </c>
+      <c r="S3" s="16" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E4" s="7" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F4" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T01",'State Market Summary'!$B$4:$B$54)</f>
@@ -6830,10 +6842,14 @@
         <f aca="false">IF(J4=0,"n/a",RANK(Q4,$Q$4:$Q$28))</f>
         <v>3</v>
       </c>
+      <c r="S4" s="30" t="n">
+        <f aca="false">IF(J4=0,4,IF(R4&lt;=7,1,IF(R4&lt;=12,2,IF(R4&lt;=19,3,4))))</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E5" s="7" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F5" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T02",'State Market Summary'!$B$4:$B$54)</f>
@@ -6883,10 +6899,14 @@
         <f aca="false">IF(J5=0,"n/a",RANK(Q5,$Q$4:$Q$28))</f>
         <v>1</v>
       </c>
+      <c r="S5" s="30" t="n">
+        <f aca="false">IF(J5=0,4,IF(R5&lt;=7,1,IF(R5&lt;=12,2,IF(R5&lt;=19,3,4))))</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E6" s="7" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F6" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T03",'State Market Summary'!$B$4:$B$54)</f>
@@ -6936,10 +6956,14 @@
         <f aca="false">IF(J6=0,"n/a",RANK(Q6,$Q$4:$Q$28))</f>
         <v>9</v>
       </c>
+      <c r="S6" s="30" t="n">
+        <f aca="false">IF(J6=0,4,IF(R6&lt;=7,1,IF(R6&lt;=12,2,IF(R6&lt;=19,3,4))))</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E7" s="7" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F7" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T04",'State Market Summary'!$B$4:$B$54)</f>
@@ -6989,10 +7013,14 @@
         <f aca="false">IF(J7=0,"n/a",RANK(Q7,$Q$4:$Q$28))</f>
         <v>11</v>
       </c>
+      <c r="S7" s="30" t="n">
+        <f aca="false">IF(J7=0,4,IF(R7&lt;=7,1,IF(R7&lt;=12,2,IF(R7&lt;=19,3,4))))</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E8" s="7" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F8" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T05",'State Market Summary'!$B$4:$B$54)</f>
@@ -7042,10 +7070,14 @@
         <f aca="false">IF(J8=0,"n/a",RANK(Q8,$Q$4:$Q$28))</f>
         <v>21</v>
       </c>
+      <c r="S8" s="30" t="n">
+        <f aca="false">IF(J8=0,4,IF(R8&lt;=7,1,IF(R8&lt;=12,2,IF(R8&lt;=19,3,4))))</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E9" s="7" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F9" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T06",'State Market Summary'!$B$4:$B$54)</f>
@@ -7095,10 +7127,14 @@
         <f aca="false">IF(J9=0,"n/a",RANK(Q9,$Q$4:$Q$28))</f>
         <v>16</v>
       </c>
+      <c r="S9" s="30" t="n">
+        <f aca="false">IF(J9=0,4,IF(R9&lt;=7,1,IF(R9&lt;=12,2,IF(R9&lt;=19,3,4))))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E10" s="7" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F10" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T07",'State Market Summary'!$B$4:$B$54)</f>
@@ -7148,10 +7184,14 @@
         <f aca="false">IF(J10=0,"n/a",RANK(Q10,$Q$4:$Q$28))</f>
         <v>8</v>
       </c>
+      <c r="S10" s="30" t="n">
+        <f aca="false">IF(J10=0,4,IF(R10&lt;=7,1,IF(R10&lt;=12,2,IF(R10&lt;=19,3,4))))</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E11" s="7" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F11" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T08",'State Market Summary'!$B$4:$B$54)</f>
@@ -7201,10 +7241,14 @@
         <f aca="false">IF(J11=0,"n/a",RANK(Q11,$Q$4:$Q$28))</f>
         <v>2</v>
       </c>
+      <c r="S11" s="30" t="n">
+        <f aca="false">IF(J11=0,4,IF(R11&lt;=7,1,IF(R11&lt;=12,2,IF(R11&lt;=19,3,4))))</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E12" s="7" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F12" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T09",'State Market Summary'!$B$4:$B$54)</f>
@@ -7254,10 +7298,14 @@
         <f aca="false">IF(J12=0,"n/a",RANK(Q12,$Q$4:$Q$28))</f>
         <v>10</v>
       </c>
+      <c r="S12" s="30" t="n">
+        <f aca="false">IF(J12=0,4,IF(R12&lt;=7,1,IF(R12&lt;=12,2,IF(R12&lt;=19,3,4))))</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E13" s="7" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F13" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T10",'State Market Summary'!$B$4:$B$54)</f>
@@ -7307,10 +7355,14 @@
         <f aca="false">IF(J13=0,"n/a",RANK(Q13,$Q$4:$Q$28))</f>
         <v>13</v>
       </c>
+      <c r="S13" s="30" t="n">
+        <f aca="false">IF(J13=0,4,IF(R13&lt;=7,1,IF(R13&lt;=12,2,IF(R13&lt;=19,3,4))))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E14" s="7" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F14" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T11",'State Market Summary'!$B$4:$B$54)</f>
@@ -7360,10 +7412,14 @@
         <f aca="false">IF(J14=0,"n/a",RANK(Q14,$Q$4:$Q$28))</f>
         <v>6</v>
       </c>
+      <c r="S14" s="30" t="n">
+        <f aca="false">IF(J14=0,4,IF(R14&lt;=7,1,IF(R14&lt;=12,2,IF(R14&lt;=19,3,4))))</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E15" s="7" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F15" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T12",'State Market Summary'!$B$4:$B$54)</f>
@@ -7413,10 +7469,14 @@
         <f aca="false">IF(J15=0,"n/a",RANK(Q15,$Q$4:$Q$28))</f>
         <v>5</v>
       </c>
+      <c r="S15" s="30" t="n">
+        <f aca="false">IF(J15=0,4,IF(R15&lt;=7,1,IF(R15&lt;=12,2,IF(R15&lt;=19,3,4))))</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E16" s="7" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F16" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T13",'State Market Summary'!$B$4:$B$54)</f>
@@ -7466,10 +7526,14 @@
         <f aca="false">IF(J16=0,"n/a",RANK(Q16,$Q$4:$Q$28))</f>
         <v>12</v>
       </c>
+      <c r="S16" s="30" t="n">
+        <f aca="false">IF(J16=0,4,IF(R16&lt;=7,1,IF(R16&lt;=12,2,IF(R16&lt;=19,3,4))))</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E17" s="7" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F17" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T14",'State Market Summary'!$B$4:$B$54)</f>
@@ -7519,10 +7583,14 @@
         <f aca="false">IF(J17=0,"n/a",RANK(Q17,$Q$4:$Q$28))</f>
         <v>15</v>
       </c>
+      <c r="S17" s="30" t="n">
+        <f aca="false">IF(J17=0,4,IF(R17&lt;=7,1,IF(R17&lt;=12,2,IF(R17&lt;=19,3,4))))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E18" s="7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F18" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T15",'State Market Summary'!$B$4:$B$54)</f>
@@ -7572,10 +7640,14 @@
         <f aca="false">IF(J18=0,"n/a",RANK(Q18,$Q$4:$Q$28))</f>
         <v>7</v>
       </c>
+      <c r="S18" s="30" t="n">
+        <f aca="false">IF(J18=0,4,IF(R18&lt;=7,1,IF(R18&lt;=12,2,IF(R18&lt;=19,3,4))))</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E19" s="7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F19" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T16",'State Market Summary'!$B$4:$B$54)</f>
@@ -7625,10 +7697,14 @@
         <f aca="false">IF(J19=0,"n/a",RANK(Q19,$Q$4:$Q$28))</f>
         <v>14</v>
       </c>
+      <c r="S19" s="30" t="n">
+        <f aca="false">IF(J19=0,4,IF(R19&lt;=7,1,IF(R19&lt;=12,2,IF(R19&lt;=19,3,4))))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E20" s="7" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F20" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T17",'State Market Summary'!$B$4:$B$54)</f>
@@ -7678,10 +7754,14 @@
         <f aca="false">IF(J20=0,"n/a",RANK(Q20,$Q$4:$Q$28))</f>
         <v>4</v>
       </c>
+      <c r="S20" s="30" t="n">
+        <f aca="false">IF(J20=0,4,IF(R20&lt;=7,1,IF(R20&lt;=12,2,IF(R20&lt;=19,3,4))))</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E21" s="7" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F21" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T18",'State Market Summary'!$B$4:$B$54)</f>
@@ -7731,10 +7811,14 @@
         <f aca="false">IF(J21=0,"n/a",RANK(Q21,$Q$4:$Q$28))</f>
         <v>20</v>
       </c>
+      <c r="S21" s="30" t="n">
+        <f aca="false">IF(J21=0,4,IF(R21&lt;=7,1,IF(R21&lt;=12,2,IF(R21&lt;=19,3,4))))</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E22" s="7" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F22" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T19",'State Market Summary'!$B$4:$B$54)</f>
@@ -7784,10 +7868,14 @@
         <f aca="false">IF(J22=0,"n/a",RANK(Q22,$Q$4:$Q$28))</f>
         <v>19</v>
       </c>
+      <c r="S22" s="30" t="n">
+        <f aca="false">IF(J22=0,4,IF(R22&lt;=7,1,IF(R22&lt;=12,2,IF(R22&lt;=19,3,4))))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E23" s="7" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F23" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T20",'State Market Summary'!$B$4:$B$54)</f>
@@ -7837,10 +7925,14 @@
         <f aca="false">IF(J23=0,"n/a",RANK(Q23,$Q$4:$Q$28))</f>
         <v>23</v>
       </c>
+      <c r="S23" s="30" t="n">
+        <f aca="false">IF(J23=0,4,IF(R23&lt;=7,1,IF(R23&lt;=12,2,IF(R23&lt;=19,3,4))))</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E24" s="7" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F24" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T21",'State Market Summary'!$B$4:$B$54)</f>
@@ -7890,10 +7982,14 @@
         <f aca="false">IF(J24=0,"n/a",RANK(Q24,$Q$4:$Q$28))</f>
         <v>18</v>
       </c>
+      <c r="S24" s="30" t="n">
+        <f aca="false">IF(J24=0,4,IF(R24&lt;=7,1,IF(R24&lt;=12,2,IF(R24&lt;=19,3,4))))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E25" s="7" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F25" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T22",'State Market Summary'!$B$4:$B$54)</f>
@@ -7943,10 +8039,14 @@
         <f aca="false">IF(J25=0,"n/a",RANK(Q25,$Q$4:$Q$28))</f>
         <v>17</v>
       </c>
+      <c r="S25" s="30" t="n">
+        <f aca="false">IF(J25=0,4,IF(R25&lt;=7,1,IF(R25&lt;=12,2,IF(R25&lt;=19,3,4))))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E26" s="7" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F26" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T23",'State Market Summary'!$B$4:$B$54)</f>
@@ -7996,10 +8096,14 @@
         <f aca="false">IF(J26=0,"n/a",RANK(Q26,$Q$4:$Q$28))</f>
         <v>22</v>
       </c>
+      <c r="S26" s="30" t="n">
+        <f aca="false">IF(J26=0,4,IF(R26&lt;=7,1,IF(R26&lt;=12,2,IF(R26&lt;=19,3,4))))</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E27" s="7" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F27" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T24",'State Market Summary'!$B$4:$B$54)</f>
@@ -8049,10 +8153,14 @@
         <f aca="false">IF(J27=0,"n/a",RANK(Q27,$Q$4:$Q$28))</f>
         <v>n/a</v>
       </c>
+      <c r="S27" s="30" t="n">
+        <f aca="false">IF(J27=0,4,IF(R27&lt;=7,1,IF(R27&lt;=12,2,IF(R27&lt;=19,3,4))))</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E28" s="7" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F28" s="8" t="n">
         <f aca="false">SUMIF('State Market Summary'!$T$4:$T$54,"T25",'State Market Summary'!$B$4:$B$54)</f>
@@ -8102,6 +8210,10 @@
         <f aca="false">IF(J28=0,"n/a",RANK(Q28,$Q$4:$Q$28))</f>
         <v>n/a</v>
       </c>
+      <c r="S28" s="30" t="n">
+        <f aca="false">IF(J28=0,4,IF(R28&lt;=7,1,IF(R28&lt;=12,2,IF(R28&lt;=19,3,4))))</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E29" s="22" t="s">
@@ -8135,7 +8247,7 @@
         <f aca="false">ROUND(G29/J29,1)</f>
         <v>209.4</v>
       </c>
-      <c r="M29" s="30" t="n">
+      <c r="M29" s="31" t="n">
         <f aca="false">H29/F29</f>
         <v>0.414561260527031</v>
       </c>
@@ -8147,7 +8259,7 @@
     </row>
     <row r="31" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E31" s="9" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>

</xml_diff>

<commit_message>
Add Academic Share definition to Kathy tab
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ysekWyVFey7vTLxxqcMoX
</commit_message>
<xml_diff>
--- a/docs/deliverables/Femasys_Territory_Plan_v4.xlsx
+++ b/docs/deliverables/Femasys_Territory_Plan_v4.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="249">
   <si>
     <t xml:space="preserve">FemaSeed U.S. Territory Plan — v4 (ALL-MD Universe, 28-Rep Hard Cap)</t>
   </si>
@@ -769,20 +769,22 @@
   </si>
   <si>
     <t xml:space="preserve">Score = min-max normalization (0-100 across staffed territories) of All MDs/Rep (20%), All Clinics/Rep (60%), Women 25-44 (10%), Median Income (10%); Education 0% (displayed, not scored). Blue cells are inputs: Reps carries the 28-rep hard-cap allocation; Women 25-44 / Median Income / Education carried from v3 Territory Plan unchanged (v3 census data-quality caveats apply). All MD/clinic counts (F-I) are sums of member states from Waterfall A rev1 labeled columns only; stray unlabeled scratch columns in the source were excluded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACADEMIC SHARE (column M) = All Academic/Group MDs / All MDs (column H / column F), both summed from Waterfall A rev1. It is the percent of a territory's total physician universe practicing in academic, hospital/system, or MSO-affiliated group settings versus private practice. Classification per the Data Request waterfall method: CMS facility IDs, hospital/system/university name tokens, and MSO rosters (incl. Unified Women's Healthcare, Axia, Privia, Pediatrix). National benchmark: 7,630 / 18,405 = 41.5%. Display only (0% score weight) - shown because access and selling motion differ materially between academic/group and private accounts. Note: metro-level academic splits are not available for the full ALL-MD universe (no row-level data exists below volume 10); metro detail is available only for the &gt;=10 tier.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="\$#,##0"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="0.0%"/>
-    <numFmt numFmtId="170" formatCode="General"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -926,7 +928,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1044,10 +1046,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6689,7 +6687,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="E1:S31"/>
+  <dimension ref="E1:S33"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20"/>
@@ -6702,7 +6700,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6842,7 +6840,7 @@
         <f aca="false">IF(J4=0,"n/a",RANK(Q4,$Q$4:$Q$28))</f>
         <v>3</v>
       </c>
-      <c r="S4" s="30" t="n">
+      <c r="S4" s="7" t="n">
         <f aca="false">IF(J4=0,4,IF(R4&lt;=7,1,IF(R4&lt;=12,2,IF(R4&lt;=19,3,4))))</f>
         <v>1</v>
       </c>
@@ -6899,7 +6897,7 @@
         <f aca="false">IF(J5=0,"n/a",RANK(Q5,$Q$4:$Q$28))</f>
         <v>1</v>
       </c>
-      <c r="S5" s="30" t="n">
+      <c r="S5" s="7" t="n">
         <f aca="false">IF(J5=0,4,IF(R5&lt;=7,1,IF(R5&lt;=12,2,IF(R5&lt;=19,3,4))))</f>
         <v>1</v>
       </c>
@@ -6956,7 +6954,7 @@
         <f aca="false">IF(J6=0,"n/a",RANK(Q6,$Q$4:$Q$28))</f>
         <v>9</v>
       </c>
-      <c r="S6" s="30" t="n">
+      <c r="S6" s="7" t="n">
         <f aca="false">IF(J6=0,4,IF(R6&lt;=7,1,IF(R6&lt;=12,2,IF(R6&lt;=19,3,4))))</f>
         <v>2</v>
       </c>
@@ -7013,7 +7011,7 @@
         <f aca="false">IF(J7=0,"n/a",RANK(Q7,$Q$4:$Q$28))</f>
         <v>11</v>
       </c>
-      <c r="S7" s="30" t="n">
+      <c r="S7" s="7" t="n">
         <f aca="false">IF(J7=0,4,IF(R7&lt;=7,1,IF(R7&lt;=12,2,IF(R7&lt;=19,3,4))))</f>
         <v>2</v>
       </c>
@@ -7070,7 +7068,7 @@
         <f aca="false">IF(J8=0,"n/a",RANK(Q8,$Q$4:$Q$28))</f>
         <v>21</v>
       </c>
-      <c r="S8" s="30" t="n">
+      <c r="S8" s="7" t="n">
         <f aca="false">IF(J8=0,4,IF(R8&lt;=7,1,IF(R8&lt;=12,2,IF(R8&lt;=19,3,4))))</f>
         <v>4</v>
       </c>
@@ -7127,7 +7125,7 @@
         <f aca="false">IF(J9=0,"n/a",RANK(Q9,$Q$4:$Q$28))</f>
         <v>16</v>
       </c>
-      <c r="S9" s="30" t="n">
+      <c r="S9" s="7" t="n">
         <f aca="false">IF(J9=0,4,IF(R9&lt;=7,1,IF(R9&lt;=12,2,IF(R9&lt;=19,3,4))))</f>
         <v>3</v>
       </c>
@@ -7184,7 +7182,7 @@
         <f aca="false">IF(J10=0,"n/a",RANK(Q10,$Q$4:$Q$28))</f>
         <v>8</v>
       </c>
-      <c r="S10" s="30" t="n">
+      <c r="S10" s="7" t="n">
         <f aca="false">IF(J10=0,4,IF(R10&lt;=7,1,IF(R10&lt;=12,2,IF(R10&lt;=19,3,4))))</f>
         <v>2</v>
       </c>
@@ -7241,7 +7239,7 @@
         <f aca="false">IF(J11=0,"n/a",RANK(Q11,$Q$4:$Q$28))</f>
         <v>2</v>
       </c>
-      <c r="S11" s="30" t="n">
+      <c r="S11" s="7" t="n">
         <f aca="false">IF(J11=0,4,IF(R11&lt;=7,1,IF(R11&lt;=12,2,IF(R11&lt;=19,3,4))))</f>
         <v>1</v>
       </c>
@@ -7298,7 +7296,7 @@
         <f aca="false">IF(J12=0,"n/a",RANK(Q12,$Q$4:$Q$28))</f>
         <v>10</v>
       </c>
-      <c r="S12" s="30" t="n">
+      <c r="S12" s="7" t="n">
         <f aca="false">IF(J12=0,4,IF(R12&lt;=7,1,IF(R12&lt;=12,2,IF(R12&lt;=19,3,4))))</f>
         <v>2</v>
       </c>
@@ -7355,7 +7353,7 @@
         <f aca="false">IF(J13=0,"n/a",RANK(Q13,$Q$4:$Q$28))</f>
         <v>13</v>
       </c>
-      <c r="S13" s="30" t="n">
+      <c r="S13" s="7" t="n">
         <f aca="false">IF(J13=0,4,IF(R13&lt;=7,1,IF(R13&lt;=12,2,IF(R13&lt;=19,3,4))))</f>
         <v>3</v>
       </c>
@@ -7412,7 +7410,7 @@
         <f aca="false">IF(J14=0,"n/a",RANK(Q14,$Q$4:$Q$28))</f>
         <v>6</v>
       </c>
-      <c r="S14" s="30" t="n">
+      <c r="S14" s="7" t="n">
         <f aca="false">IF(J14=0,4,IF(R14&lt;=7,1,IF(R14&lt;=12,2,IF(R14&lt;=19,3,4))))</f>
         <v>1</v>
       </c>
@@ -7469,7 +7467,7 @@
         <f aca="false">IF(J15=0,"n/a",RANK(Q15,$Q$4:$Q$28))</f>
         <v>5</v>
       </c>
-      <c r="S15" s="30" t="n">
+      <c r="S15" s="7" t="n">
         <f aca="false">IF(J15=0,4,IF(R15&lt;=7,1,IF(R15&lt;=12,2,IF(R15&lt;=19,3,4))))</f>
         <v>1</v>
       </c>
@@ -7526,7 +7524,7 @@
         <f aca="false">IF(J16=0,"n/a",RANK(Q16,$Q$4:$Q$28))</f>
         <v>12</v>
       </c>
-      <c r="S16" s="30" t="n">
+      <c r="S16" s="7" t="n">
         <f aca="false">IF(J16=0,4,IF(R16&lt;=7,1,IF(R16&lt;=12,2,IF(R16&lt;=19,3,4))))</f>
         <v>2</v>
       </c>
@@ -7583,7 +7581,7 @@
         <f aca="false">IF(J17=0,"n/a",RANK(Q17,$Q$4:$Q$28))</f>
         <v>15</v>
       </c>
-      <c r="S17" s="30" t="n">
+      <c r="S17" s="7" t="n">
         <f aca="false">IF(J17=0,4,IF(R17&lt;=7,1,IF(R17&lt;=12,2,IF(R17&lt;=19,3,4))))</f>
         <v>3</v>
       </c>
@@ -7640,7 +7638,7 @@
         <f aca="false">IF(J18=0,"n/a",RANK(Q18,$Q$4:$Q$28))</f>
         <v>7</v>
       </c>
-      <c r="S18" s="30" t="n">
+      <c r="S18" s="7" t="n">
         <f aca="false">IF(J18=0,4,IF(R18&lt;=7,1,IF(R18&lt;=12,2,IF(R18&lt;=19,3,4))))</f>
         <v>1</v>
       </c>
@@ -7697,7 +7695,7 @@
         <f aca="false">IF(J19=0,"n/a",RANK(Q19,$Q$4:$Q$28))</f>
         <v>14</v>
       </c>
-      <c r="S19" s="30" t="n">
+      <c r="S19" s="7" t="n">
         <f aca="false">IF(J19=0,4,IF(R19&lt;=7,1,IF(R19&lt;=12,2,IF(R19&lt;=19,3,4))))</f>
         <v>3</v>
       </c>
@@ -7754,7 +7752,7 @@
         <f aca="false">IF(J20=0,"n/a",RANK(Q20,$Q$4:$Q$28))</f>
         <v>4</v>
       </c>
-      <c r="S20" s="30" t="n">
+      <c r="S20" s="7" t="n">
         <f aca="false">IF(J20=0,4,IF(R20&lt;=7,1,IF(R20&lt;=12,2,IF(R20&lt;=19,3,4))))</f>
         <v>1</v>
       </c>
@@ -7811,7 +7809,7 @@
         <f aca="false">IF(J21=0,"n/a",RANK(Q21,$Q$4:$Q$28))</f>
         <v>20</v>
       </c>
-      <c r="S21" s="30" t="n">
+      <c r="S21" s="7" t="n">
         <f aca="false">IF(J21=0,4,IF(R21&lt;=7,1,IF(R21&lt;=12,2,IF(R21&lt;=19,3,4))))</f>
         <v>4</v>
       </c>
@@ -7868,7 +7866,7 @@
         <f aca="false">IF(J22=0,"n/a",RANK(Q22,$Q$4:$Q$28))</f>
         <v>19</v>
       </c>
-      <c r="S22" s="30" t="n">
+      <c r="S22" s="7" t="n">
         <f aca="false">IF(J22=0,4,IF(R22&lt;=7,1,IF(R22&lt;=12,2,IF(R22&lt;=19,3,4))))</f>
         <v>3</v>
       </c>
@@ -7925,7 +7923,7 @@
         <f aca="false">IF(J23=0,"n/a",RANK(Q23,$Q$4:$Q$28))</f>
         <v>23</v>
       </c>
-      <c r="S23" s="30" t="n">
+      <c r="S23" s="7" t="n">
         <f aca="false">IF(J23=0,4,IF(R23&lt;=7,1,IF(R23&lt;=12,2,IF(R23&lt;=19,3,4))))</f>
         <v>4</v>
       </c>
@@ -7982,7 +7980,7 @@
         <f aca="false">IF(J24=0,"n/a",RANK(Q24,$Q$4:$Q$28))</f>
         <v>18</v>
       </c>
-      <c r="S24" s="30" t="n">
+      <c r="S24" s="7" t="n">
         <f aca="false">IF(J24=0,4,IF(R24&lt;=7,1,IF(R24&lt;=12,2,IF(R24&lt;=19,3,4))))</f>
         <v>3</v>
       </c>
@@ -8039,7 +8037,7 @@
         <f aca="false">IF(J25=0,"n/a",RANK(Q25,$Q$4:$Q$28))</f>
         <v>17</v>
       </c>
-      <c r="S25" s="30" t="n">
+      <c r="S25" s="7" t="n">
         <f aca="false">IF(J25=0,4,IF(R25&lt;=7,1,IF(R25&lt;=12,2,IF(R25&lt;=19,3,4))))</f>
         <v>3</v>
       </c>
@@ -8096,7 +8094,7 @@
         <f aca="false">IF(J26=0,"n/a",RANK(Q26,$Q$4:$Q$28))</f>
         <v>22</v>
       </c>
-      <c r="S26" s="30" t="n">
+      <c r="S26" s="7" t="n">
         <f aca="false">IF(J26=0,4,IF(R26&lt;=7,1,IF(R26&lt;=12,2,IF(R26&lt;=19,3,4))))</f>
         <v>4</v>
       </c>
@@ -8153,7 +8151,7 @@
         <f aca="false">IF(J27=0,"n/a",RANK(Q27,$Q$4:$Q$28))</f>
         <v>n/a</v>
       </c>
-      <c r="S27" s="30" t="n">
+      <c r="S27" s="7" t="n">
         <f aca="false">IF(J27=0,4,IF(R27&lt;=7,1,IF(R27&lt;=12,2,IF(R27&lt;=19,3,4))))</f>
         <v>4</v>
       </c>
@@ -8210,7 +8208,7 @@
         <f aca="false">IF(J28=0,"n/a",RANK(Q28,$Q$4:$Q$28))</f>
         <v>n/a</v>
       </c>
-      <c r="S28" s="30" t="n">
+      <c r="S28" s="7" t="n">
         <f aca="false">IF(J28=0,4,IF(R28&lt;=7,1,IF(R28&lt;=12,2,IF(R28&lt;=19,3,4))))</f>
         <v>4</v>
       </c>
@@ -8247,7 +8245,7 @@
         <f aca="false">ROUND(G29/J29,1)</f>
         <v>209.4</v>
       </c>
-      <c r="M29" s="31" t="n">
+      <c r="M29" s="30" t="n">
         <f aca="false">H29/F29</f>
         <v>0.414561260527031</v>
       </c>
@@ -8275,10 +8273,29 @@
       <c r="Q31" s="9"/>
       <c r="R31" s="9"/>
     </row>
+    <row r="33" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E33" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="E1:R1"/>
     <mergeCell ref="E31:R31"/>
+    <mergeCell ref="E33:R33"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>